<commit_message>
Ajuste script de IVA + Conta Razão - Validado
</commit_message>
<xml_diff>
--- a/Planilhas/Pedidos.xlsx
+++ b/Planilhas/Pedidos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junio\OneDrive\Área de Trabalho\Documentos\Scripts Github\automations\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABEB8E9A-82EB-4450-9E02-0D1E010F3908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB238E02-C775-4C0C-96D3-276DE407678A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{B22F4247-8A78-4CA2-917D-234C68224E18}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B22F4247-8A78-4CA2-917D-234C68224E18}"/>
   </bookViews>
   <sheets>
     <sheet name="ALTERAR PARA F5" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -53,10 +42,10 @@
     <t>Modo</t>
   </si>
   <si>
-    <t>AMBOS</t>
+    <t>F4</t>
   </si>
   <si>
-    <t>F4</t>
+    <t>RAZAO</t>
   </si>
 </sst>
 </file>
@@ -67,19 +56,19 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -229,39 +218,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -313,7 +302,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -424,6 +413,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -432,13 +428,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -503,31 +492,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -536,16 +505,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C176DAE8-01D4-4562-9DC5-3FF54C0846F5}">
   <dimension ref="A1:E62"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.90625" customWidth="1"/>
-    <col min="4" max="4" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -562,7 +531,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>4500030627</v>
       </c>
@@ -570,16 +539,16 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>3201010111</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>4500030628</v>
       </c>
@@ -587,16 +556,16 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3">
         <v>3201010111</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4500030629</v>
       </c>
@@ -604,16 +573,16 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>3201010111</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4500030630</v>
       </c>
@@ -621,16 +590,16 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>3201010111</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4500030631</v>
       </c>
@@ -638,16 +607,16 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6">
         <v>3201010111</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4500030632</v>
       </c>
@@ -655,16 +624,16 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>3201010111</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4500030633</v>
       </c>
@@ -672,16 +641,16 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>3201010111</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4500030634</v>
       </c>
@@ -689,16 +658,16 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>3201010111</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4500030635</v>
       </c>
@@ -706,16 +675,16 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D10">
         <v>3201010111</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4500030638</v>
       </c>
@@ -723,16 +692,16 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>3201010111</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>4500030639</v>
       </c>
@@ -740,16 +709,16 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D12">
         <v>3201010111</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>4500030640</v>
       </c>
@@ -757,16 +726,16 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>3201010111</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>4500030641</v>
       </c>
@@ -774,16 +743,16 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>3201010111</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>4500030642</v>
       </c>
@@ -791,16 +760,16 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>3201010111</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>4500030643</v>
       </c>
@@ -808,16 +777,16 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16">
         <v>3201010111</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>4500030646</v>
       </c>
@@ -825,16 +794,16 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D17">
         <v>3201010111</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4500030647</v>
       </c>
@@ -842,16 +811,16 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>3201010111</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>4500030648</v>
       </c>
@@ -859,16 +828,16 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D19">
         <v>3201010111</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>4500030649</v>
       </c>
@@ -876,16 +845,16 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D20">
         <v>3201010111</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>4500030650</v>
       </c>
@@ -893,16 +862,16 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21">
         <v>3201010111</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>4500030651</v>
       </c>
@@ -910,16 +879,16 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22">
         <v>3201010111</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>4500030652</v>
       </c>
@@ -927,16 +896,16 @@
         <v>10</v>
       </c>
       <c r="C23" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23">
         <v>3201010111</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>4500030653</v>
       </c>
@@ -944,16 +913,16 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D24">
         <v>3201010111</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>4500030656</v>
       </c>
@@ -961,16 +930,16 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25">
         <v>3201010111</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>4500030657</v>
       </c>
@@ -978,16 +947,16 @@
         <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26">
         <v>3201010111</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>4500030671</v>
       </c>
@@ -995,16 +964,16 @@
         <v>10</v>
       </c>
       <c r="C27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D27">
         <v>3201010111</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>4500030672</v>
       </c>
@@ -1012,16 +981,16 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28">
         <v>3201010111</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>4500030673</v>
       </c>
@@ -1029,16 +998,16 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D29">
         <v>3201010111</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4500030674</v>
       </c>
@@ -1046,16 +1015,16 @@
         <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D30">
         <v>3201010111</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>4500030675</v>
       </c>
@@ -1063,16 +1032,16 @@
         <v>10</v>
       </c>
       <c r="C31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D31">
         <v>3201010111</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>4500030676</v>
       </c>
@@ -1080,16 +1049,16 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D32">
         <v>3201010111</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>4500030677</v>
       </c>
@@ -1097,16 +1066,16 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D33">
         <v>3201010111</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>4500030678</v>
       </c>
@@ -1114,16 +1083,16 @@
         <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D34">
         <v>3201010111</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>4500030679</v>
       </c>
@@ -1131,16 +1100,16 @@
         <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D35">
         <v>3201010111</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>4500030680</v>
       </c>
@@ -1148,16 +1117,16 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D36">
         <v>3201010111</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>4500030681</v>
       </c>
@@ -1165,16 +1134,16 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D37">
         <v>3201010111</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>4500030682</v>
       </c>
@@ -1182,16 +1151,16 @@
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D38">
         <v>3201010111</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>4500030683</v>
       </c>
@@ -1199,16 +1168,16 @@
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D39">
         <v>3201010111</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>4500030684</v>
       </c>
@@ -1216,16 +1185,16 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D40">
         <v>3201010111</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>4500030685</v>
       </c>
@@ -1233,16 +1202,16 @@
         <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D41">
         <v>3201010111</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>4500030686</v>
       </c>
@@ -1250,16 +1219,16 @@
         <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D42">
         <v>3201010111</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>4500030687</v>
       </c>
@@ -1267,16 +1236,16 @@
         <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D43">
         <v>3201010111</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>4500030688</v>
       </c>
@@ -1284,16 +1253,16 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D44">
         <v>3201010111</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>4500030689</v>
       </c>
@@ -1301,16 +1270,16 @@
         <v>10</v>
       </c>
       <c r="C45" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D45">
         <v>3201010111</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>4500030690</v>
       </c>
@@ -1318,16 +1287,16 @@
         <v>10</v>
       </c>
       <c r="C46" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D46">
         <v>3201010111</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>4500030692</v>
       </c>
@@ -1335,16 +1304,16 @@
         <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47">
         <v>3201010111</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>4500030693</v>
       </c>
@@ -1352,16 +1321,16 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D48">
         <v>3201010111</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>4500030694</v>
       </c>
@@ -1369,16 +1338,16 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49">
         <v>3201010111</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>4500030695</v>
       </c>
@@ -1386,16 +1355,16 @@
         <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D50">
         <v>3201010111</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>4500030715</v>
       </c>
@@ -1403,16 +1372,16 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D51">
         <v>3201010111</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>4500030716</v>
       </c>
@@ -1420,16 +1389,16 @@
         <v>10</v>
       </c>
       <c r="C52" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D52">
         <v>3201010111</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>4500030717</v>
       </c>
@@ -1437,16 +1406,16 @@
         <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D53">
         <v>3201010111</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>4500030718</v>
       </c>
@@ -1454,16 +1423,16 @@
         <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D54">
         <v>3201010111</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>4500030720</v>
       </c>
@@ -1471,16 +1440,16 @@
         <v>10</v>
       </c>
       <c r="C55" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D55">
         <v>3201010111</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>4500030721</v>
       </c>
@@ -1488,16 +1457,16 @@
         <v>10</v>
       </c>
       <c r="C56" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D56">
         <v>3201010111</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>4500030722</v>
       </c>
@@ -1505,16 +1474,16 @@
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D57">
         <v>3201010111</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>4500030723</v>
       </c>
@@ -1522,16 +1491,16 @@
         <v>10</v>
       </c>
       <c r="C58" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D58">
         <v>3201010111</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>4500030724</v>
       </c>
@@ -1539,16 +1508,16 @@
         <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D59">
         <v>3201010111</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>4500030725</v>
       </c>
@@ -1556,16 +1525,16 @@
         <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D60">
         <v>3201010111</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>4500030726</v>
       </c>
@@ -1573,16 +1542,16 @@
         <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D61">
         <v>3201010111</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>4500030727</v>
       </c>
@@ -1590,13 +1559,13 @@
         <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D62">
         <v>3201010111</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>